<commit_message>
Added Files to project 3. Corrections made to projects 1 and 2
</commit_message>
<xml_diff>
--- a/project-01-ai-system-inventory/ai-system-inventory-signalpath.xlsx
+++ b/project-01-ai-system-inventory/ai-system-inventory-signalpath.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonat\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/deaf463e8039491e/Documents/GitHub/AiGovernance/project-01-ai-system-inventory/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB2117CA-A4D3-4BA7-972E-53D920389F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{BB2117CA-A4D3-4BA7-972E-53D920389F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{891C488A-7057-4804-B187-11F93AFF8FBE}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10050" yWindow="-32520" windowWidth="57840" windowHeight="31920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ai-system-inventory" sheetId="1" r:id="rId1"/>
@@ -213,15 +213,9 @@
     <t>SP-AI-004</t>
   </si>
   <si>
-    <t>CaptionCall AI</t>
-  </si>
-  <si>
     <t>AI-powered home phone captioning service displaying real-time captions of phone conversations on a screen device for hard-of-hearing users.</t>
   </si>
   <si>
-    <t>CaptionCall Product Line</t>
-  </si>
-  <si>
     <t>Captioned telephone service for hard-of-hearing home users</t>
   </si>
   <si>
@@ -231,9 +225,6 @@
     <t>Real-time caption display on device screen</t>
   </si>
   <si>
-    <t>Head of Product — CaptionCall</t>
-  </si>
-  <si>
     <t>Hard-of-hearing home phone users</t>
   </si>
   <si>
@@ -697,6 +688,15 @@
   </si>
   <si>
     <t>CRITICAL. This is not a hypothetical risk — shadow AI adoption is active in every organisation of this size. Interpreter coordinators summarising call logs in ChatGPT. Legal staff uploading contracts to Claude. Engineers pasting API schemas into Gemini. Discovery required immediately. Policy, training, and approved-tool list needed before this inventory is presented to the board.</t>
+  </si>
+  <si>
+    <t>SignalPath CaptionLine</t>
+  </si>
+  <si>
+    <t>CaptionLine Product Line</t>
+  </si>
+  <si>
+    <t>Head of Product — CaptionLine</t>
   </si>
 </sst>
 </file>
@@ -1331,90 +1331,90 @@
         <v>61</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>20</v>
       </c>
       <c r="E5" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>41</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>68</v>
+        <v>223</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>43</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="N5" s="7" t="s">
         <v>46</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="E6" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="G6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="H6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="I6" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="J6" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="K6" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="L6" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="L6" s="8" t="s">
-        <v>85</v>
       </c>
       <c r="M6" s="8" t="s">
         <v>45</v>
@@ -1426,48 +1426,48 @@
         <v>47</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="E7" s="8" t="s">
+      <c r="H7" s="3" t="s">
         <v>91</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>41</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L7" s="8" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="M7" s="8" t="s">
         <v>45</v>
@@ -1479,36 +1479,36 @@
         <v>47</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8" s="8" t="s">
+      <c r="H8" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>106</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>41</v>
@@ -1517,10 +1517,10 @@
         <v>57</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="M8" s="8" t="s">
         <v>45</v>
@@ -1532,48 +1532,48 @@
         <v>47</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="E9" s="8" t="s">
+      <c r="H9" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>117</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>41</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="M9" s="8" t="s">
         <v>45</v>
@@ -1582,160 +1582,160 @@
         <v>46</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" s="8" t="s">
+      <c r="H10" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>41</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="M10" s="8" t="s">
         <v>45</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="O10" s="8" t="s">
         <v>47</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="E11" s="8" t="s">
+      <c r="H11" s="3" t="s">
         <v>139</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>142</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>41</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="M11" s="8" t="s">
         <v>45</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="E12" s="8" t="s">
+      <c r="H12" s="3" t="s">
         <v>151</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>154</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>41</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="L12" s="8" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="M12" s="8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="N12" s="8" t="s">
         <v>46</v>
@@ -1744,101 +1744,101 @@
         <v>47</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="E13" s="8" t="s">
+      <c r="H13" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="I13" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="J13" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="K13" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="L13" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="L13" s="8" t="s">
-        <v>169</v>
       </c>
       <c r="M13" s="8" t="s">
         <v>45</v>
       </c>
       <c r="N13" s="8" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="O13" s="8" t="s">
         <v>47</v>
       </c>
       <c r="P13" s="3" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="Q13" s="3" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="E14" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="G14" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="H14" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="I14" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="J14" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="K14" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="I14" s="9" t="s">
+      <c r="L14" s="9" t="s">
         <v>179</v>
-      </c>
-      <c r="J14" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="K14" s="9" t="s">
-        <v>181</v>
-      </c>
-      <c r="L14" s="9" t="s">
-        <v>182</v>
       </c>
       <c r="M14" s="9" t="s">
         <v>45</v>
@@ -1850,101 +1850,101 @@
         <v>31</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="Q14" s="4" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="E15" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="F15" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="G15" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="H15" s="5" t="s">
         <v>189</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>192</v>
       </c>
       <c r="I15" s="10" t="s">
         <v>41</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="O15" s="10" t="s">
         <v>47</v>
       </c>
       <c r="P15" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="F16" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="G16" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="D16" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="E16" s="10" t="s">
+      <c r="H16" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>204</v>
       </c>
       <c r="I16" s="10" t="s">
         <v>41</v>
       </c>
       <c r="J16" s="10" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="M16" s="10" t="s">
         <v>45</v>
@@ -1953,66 +1953,66 @@
         <v>46</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="P16" s="5" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Q16" s="5" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="251" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D17" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="E17" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="G17" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="H17" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="E17" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="F17" s="6" t="s">
+      <c r="I17" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="J17" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="K17" s="11" t="s">
         <v>215</v>
       </c>
-      <c r="I17" s="11" t="s">
+      <c r="L17" s="11" t="s">
         <v>216</v>
       </c>
-      <c r="J17" s="11" t="s">
+      <c r="M17" s="11" t="s">
         <v>217</v>
-      </c>
-      <c r="K17" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="L17" s="11" t="s">
-        <v>219</v>
-      </c>
-      <c r="M17" s="11" t="s">
-        <v>220</v>
       </c>
       <c r="N17" s="11" t="s">
         <v>30</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="P17" s="6" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>